<commit_message>
deploy: add local one-click bootstrap
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -227,7 +227,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>feature/taoyuan-production-readiness</t>
+          <t>codex/tencent-cloud-deploy -&gt; main</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>目标组合档通过：ok .../tests/stress 1.701s</t>
+          <t>目标组合档通过：ok .../tests/stress 7.040s</t>
         </is>
       </c>
     </row>
@@ -2471,66 +2471,83 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>k6 负载脚本</t>
+          <t>本地一键部署</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>tests/load/*.k6.js</t>
+          <t>scripts/deploy/local-one-click.sh</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>基线通过，auth/admin 重压边界已记录</t>
+          <t>初始化 SQLite、演示用户、管理员并自动选择空闲端口</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>浏览器视觉审查</t>
+          <t>k6 负载脚本</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>tmp/visual-review/*.png</t>
+          <t>tests/load/*.k6.js</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>已捕获桌面/移动、用户页、充值页和后台页；22 张截图，0 破图/溢出/控制台错误</t>
+          <t>基线通过，auth/admin 重压边界已记录</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>浏览器视觉审查</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>E2E_BASE_URL=http://127.0.0.1:18080 npx playwright test</t>
+          <t>tmp/visual-review/*.png</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>通过，31/31</t>
+          <t>已捕获桌面/移动、用户页、充值页和后台页；22 张截图，0 破图/溢出/控制台错误</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Playwright E2E</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>cd e2e &amp;&amp; npx playwright test</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>通过，29/29</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>CI/CD</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>.github/workflows/ci.yml</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>workflow 已新增，远端运行待 push 后确认</t>
         </is>

</xml_diff>

<commit_message>
docs: finalize submission package and readiness fixes
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -4,7 +4,8 @@
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
     <sheet name="Test Cases" sheetId="2" r:id="rId2"/>
-    <sheet name="Verification" sheetId="3" r:id="rId3"/>
+    <sheet name="Seed Samples" sheetId="3" r:id="rId3"/>
+    <sheet name="Verification" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -172,13 +173,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>来源</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>docs/generated/app-test-cases.csv</t>
-        </is>
+          <t>样例旅程总数</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>12</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -187,22 +186,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Route</t>
-        </is>
-      </c>
-      <c r="E5">
-        <v>23</v>
+          <t/>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>生成方式</t>
+          <t>来源</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>由代码路由、schema、测试文件生成后汇总</t>
+          <t>docs/generated/app-test-cases.csv</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -212,35 +213,87 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="E6">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>样例数据来源</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>docs/generated/sample-journeys.csv</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E7">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>生成方式</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>由代码路由、schema、seed、测试文件生成后汇总</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>适用分支</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>codex/tencent-cloud-deploy -&gt; main</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2347,96 +2400,1055 @@
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="24" customWidth="1"/>
+    <col min="12" max="12" width="24" customWidth="1"/>
+    <col min="13" max="13" width="24" customWidth="1"/>
+    <col min="14" max="14" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t>验证项</t>
+          <t>slug</t>
         </is>
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
-          <t>命令或证据</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
-          <t>当前状态</t>
+          <t>subtitle</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>fantasy_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t>visual_style</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>adventure_index</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t>obscurity_level</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t>risk_level</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t>image_path</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t>story_hook</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t>mbti</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>生成图表/矩阵</t>
+          <t>bolivia-salt-flat-trek</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>python3 scripts/docs/generate_project_artifacts.py</t>
+          <t>徒步穿越玻利维亚盐沼</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>通过，docs/generated/* 已生成</t>
+          <t>世界尽头的镜面，你踩碎了天空</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>南美洲 · 玻利维亚</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>solitude</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>surreal</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>15999</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>bolivia-salt-flat.jpg</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>你踩碎了天空，世界失去了边界</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>solitude;visual;hidden</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>INFP:5;ISFJ:4;INFJ:4</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr" s="1">
         <is>
-          <t>Go 单元/集成测试</t>
+          <t>iceland-lava-tunnel-cycling</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="1">
         <is>
-          <t>go test ./...</t>
+          <t>冰岛熔岩隧道骑行</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>通过</t>
+          <t>地球内部有一条路，只有你知道</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="1">
+        <is>
+          <t>欧洲 · 冰岛</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="1">
+        <is>
+          <t>extreme</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="1">
+        <is>
+          <t>dramatic</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr" s="1">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr" s="1">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr" s="1">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr" s="1">
+        <is>
+          <t>19999</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr" s="1">
+        <is>
+          <t>iceland-lava-tunnel.jpg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr" s="1">
+        <is>
+          <t>地球内部有一条路，只有你知道</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr" s="1">
+        <is>
+          <t>extreme;hidden;nature</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr" s="1">
+        <is>
+          <t>INTJ:5;ENTP:4;ISTP:4</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Go vet</t>
+          <t>japan-onsen-temple-meditation</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>go vet ./...</t>
+          <t>日本秘境温泉寺庙冥想</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>通过</t>
+          <t>凌晨三点，只有蒸汽和沉默</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>亚洲 · 日本</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>spiritual</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>8999</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>japan-temple-onsen.jpg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>凌晨三点，只有蒸汽和沉默</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>solitude;culture;spiritual</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>INFP:5;ISFJ:5;INFJ:4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JS 语法检查</t>
+          <t>morocco-sahara-camel-camp</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>find web/js -name '*.js' -exec node --check {} \;</t>
+          <t>摩洛哥撒哈拉沙漠骆驼夜宿</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>通过</t>
+          <t>没有光污染的天空，让人害怕的辽阔</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>非洲 · 摩洛哥</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>dramatic</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>12999</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>morocco-sahara-camp.jpg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>没有光污染的天空，让人害怕的辽阔</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>visual;nature;night</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>ENFP:5;ESFP:4;ENFJ:4</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>greenland-dog-sled-solo</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>格陵兰犬拉雪橇独行</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>零下三十度，全世界只有你和十二条狗</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>北极 · 格陵兰</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>extreme</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>29999</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>greenland-dog-sled.jpg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>零下三十度，全世界只有你和十二条狗</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>extreme;solitude;nature</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>ESTP:5;ENTJ:4;ISTP:4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>norway-aurora-hunt</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>挪威特罗姆瑟极光狩猎</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>在零下二十度的黑夜里，等一束来自太阳的光</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>欧洲 · 挪威</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>dramatic</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>18999</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>norway-aurora.jpg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>在零下二十度的黑夜里，等一束来自太阳的光</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>visual;nature;night</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>INFP:5;ISFJ:4;INFJ:5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>new-zealand-milford-kayak</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>新西兰米尔福德峡湾皮划艇</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>在两千米高的瀑布下，你渺小得像一滴水</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>大洋洲 · 新西兰</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>extreme</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>22999</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>new-zealand-milford.jpg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>在两千米高的瀑布下，你渺小得像一滴水</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>extreme;visual;nature</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>ENTP:4;ESTP:5;ISTP:5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>patagonia-torres-del-paine-trek</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>巴塔哥尼亚百内国家公园徒步</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>狂风把云撕碎，露出花岗岩的尖顶</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>南美洲 · 智利</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>extreme</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>dramatic</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>24999</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>patagonia-torres-del-paine.jpg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>狂风把云撕碎，露出花岗岩的尖顶</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>extreme;hidden;nature</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>INTJ:5;ISTJ:4;ENTJ:5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>turkey-cappadocia-balloon</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>土耳其卡帕多西亚热气球日出</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>一百个热气球同时升空，你漂浮在月球表面</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>亚洲 · 土耳其</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>visual</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>surreal</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>16999</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>turkey-cappadocia.jpg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>一百个热气球同时升空，你漂浮在月球表面</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>visual;culture;night</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>ENFP:5;ISFP:4;ESFP:5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>peru-machu-picchu-inca-trail</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>秘鲁马丘比丘印加古道徒步</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>四天三夜，走在五百年前铺好的石阶上</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>南美洲 · 秘鲁</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>culture</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>21999</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>peru-machu-picchu.jpg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>四天三夜，走在五百年前铺好的石阶上</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>extreme;culture;hidden</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>ISFJ:5;ISTJ:5;INFJ:4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>namibia-deadvlei-stars</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>纳米比亚死亡谷星空露营</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>九百年的枯树站在红沙丘上，像大地竖起的图腾</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>非洲 · 纳米比亚</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>surreal</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>19999</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>namibia-deadvlei.jpg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>九百年的枯树站在红沙丘上，像大地竖起的图腾</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>visual;nature;night</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>INFP:5;INTJ:4;INFJ:5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>maldives-underwater-dining</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>马尔代夫海底餐厅晚宴</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>在五米深的海底，和鲨鱼一起享用香槟</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>亚洲 · 马尔代夫</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>visual</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>surreal</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>35999</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>maldives-underwater.jpg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>在五米深的海底，和鲨鱼一起享用香槟</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>visual;culture;hidden</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>ISFJ:4;ESFJ:5;ENFJ:5</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>验证项</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t>命令或证据</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>当前状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>生成图表/矩阵</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>python3 scripts/docs/generate_project_artifacts.py</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>通过，docs/generated/* 已生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr" s="1">
+        <is>
+          <t>Go 单元/集成测试</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="1">
+        <is>
+          <t>go test ./...</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="1">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Go vet</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>go vet ./...</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>JS 语法检查</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>find web/js -name '*.js' -exec node --check {} \;</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>Go stress</t>
         </is>
       </c>
@@ -2447,7 +3459,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>目标组合档通过：ok .../tests/stress 7.040s</t>
+          <t>目标组合档通过：ok .../tests/stress 1.660s</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: expand sample journey data export
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -2411,75 +2411,99 @@
     <col min="12" max="12" width="24" customWidth="1"/>
     <col min="13" max="13" width="24" customWidth="1"/>
     <col min="14" max="14" width="24" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
+    <col min="16" max="16" width="24" customWidth="1"/>
+    <col min="17" max="17" width="24" customWidth="1"/>
+    <col min="18" max="18" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t>subtitle</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>story_hook</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t>fantasy_type</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
         <is>
           <t>visual_style</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="1">
         <is>
           <t>adventure_index</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="K1" t="inlineStr" s="1">
         <is>
           <t>obscurity_level</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="L1" t="inlineStr" s="1">
         <is>
           <t>risk_level</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t>mood_keywords</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="O1" t="inlineStr" s="1">
         <is>
           <t>image_path</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="1">
-        <is>
-          <t>story_hook</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr" s="1">
+      <c r="P1" t="inlineStr" s="1">
+        <is>
+          <t>booking_url</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr" s="1">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr" s="1">
+      <c r="R1" t="inlineStr" s="1">
         <is>
           <t>mbti</t>
         </is>
@@ -2488,864 +2512,1104 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>bolivia-salt-flat-trek</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>徒步穿越玻利维亚盐沼</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>世界尽头的镜面，你踩碎了天空</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>你踩碎了天空，世界失去了边界</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>当雨季薄水覆盖乌尤尼盐沼，整个世界失去了边界。你踩着半厘米深的水，脚下是天空，头上也是天空。没有地平线，没有方向感，只有绵延至无穷远的白色寂静。这不是旅行，这是一次关于孤独和无限的哲学实验。</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>南美洲 · 玻利维亚</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>solitude</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>surreal</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>["孤独";"无限感";"镜面世界";"极简主义"]</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>15999</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>bolivia-salt-flat.jpg</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>你踩碎了天空，世界失去了边界</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>solitude;visual;hidden</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>INFP:5;ISFJ:4;INFJ:4</t>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>孤独感(solitude);视觉奇观(visual);隐秘小众(hidden)</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>INFP-调停者:5;ISFJ-守护者:4;INFJ-提倡者:4</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr" s="1">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="1">
+        <is>
           <t>iceland-lava-tunnel-cycling</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr" s="1">
+      <c r="C3" t="inlineStr" s="1">
         <is>
           <t>冰岛熔岩隧道骑行</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="1">
+      <c r="D3" t="inlineStr" s="1">
         <is>
           <t>地球内部有一条路，只有你知道</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="1">
+      <c r="E3" t="inlineStr" s="1">
+        <is>
+          <t>地球内部有一条路，只有你知道</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="1">
+        <is>
+          <t>斯奈山半岛深处，一条形成于三千年前的熔岩隧道蜿蜒数公里。没有游客，没有指示牌，只有你的头灯照亮的玄武岩壁和远处永恒的黑暗。每次踩踏，回声在洞穴里反复叠加，像是地球本身在对你低语。</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr" s="1">
         <is>
           <t>欧洲 · 冰岛</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr" s="1">
+      <c r="H3" t="inlineStr" s="1">
         <is>
           <t>extreme</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr" s="1">
+      <c r="I3" t="inlineStr" s="1">
         <is>
           <t>dramatic</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr" s="1">
+      <c r="J3" t="inlineStr" s="1">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr" s="1">
+      <c r="K3" t="inlineStr" s="1">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr" s="1">
+      <c r="L3" t="inlineStr" s="1">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr" s="1">
+      <c r="M3" t="inlineStr" s="1">
+        <is>
+          <t>["黑暗";"回声";"原始";"恐惧";"自由"]</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr" s="1">
         <is>
           <t>19999</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr" s="1">
+      <c r="O3" t="inlineStr" s="1">
         <is>
           <t>iceland-lava-tunnel.jpg</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr" s="1">
-        <is>
-          <t>地球内部有一条路，只有你知道</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr" s="1">
-        <is>
-          <t>extreme;hidden;nature</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr" s="1">
-        <is>
-          <t>INTJ:5;ENTP:4;ISTP:4</t>
+      <c r="P3" t="inlineStr" s="1">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr" s="1">
+        <is>
+          <t>极限挑战(extreme);隐秘小众(hidden);自然原始(nature)</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr" s="1">
+        <is>
+          <t>INTJ-建筑师:5;ENTP-辩论家:4;ISTP-鉴赏家:4</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>japan-onsen-temple-meditation</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>日本秘境温泉寺庙冥想</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>凌晨三点，只有蒸汽和沉默</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>凌晨三点，只有蒸汽和沉默</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>和歌山山中的某座小寺，接受在家居士入住。凌晨三点随僧侣起床，在黑暗中徒步至山顶，看第一缕日光穿透云海。之后是两小时的无声冥想，浸泡在寺院后山的天然温泉里，感受水温与思绪同时冷却。</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>亚洲 · 日本</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>spiritual</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>["冥想";"沉默";"蒸汽";"冷却";"纯净"]</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>8999</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>japan-temple-onsen.jpg</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>凌晨三点，只有蒸汽和沉默</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>solitude;culture;spiritual</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>INFP:5;ISFJ:5;INFJ:4</t>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>孤独感(solitude);文化沉浸(culture);精神体验(spiritual)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>INFP-调停者:5;ISFJ-守护者:5;INFJ-提倡者:4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>morocco-sahara-camel-camp</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>摩洛哥撒哈拉沙漠骆驼夜宿</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>没有光污染的天空，让人害怕的辽阔</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>没有光污染的天空，让人害怕的辽阔</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>梅尔祖卡的沙丘没有截止时间。骑着骆驼进入沙漠腹地三小时，在一个没有任何人工光源的地方支起帐篷。当银河从地平线一端铺至另一端，你突然理解了古代游牧民为何相信神住在天上——那里比地面上任何地方都更像一个家。</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>非洲 · 摩洛哥</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>dramatic</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>["星空";"辽阔";"游牧";"银河";"夜晚"]</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>12999</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>morocco-sahara-camp.jpg</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>没有光污染的天空，让人害怕的辽阔</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>visual;nature;night</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>ENFP:5;ESFP:4;ENFJ:4</t>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>视觉奇观(visual);自然原始(nature);夜晚魔法(night)</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>ENFP-竞选者:5;ESFP-表演者:4;ENFJ-主人公:4</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>greenland-dog-sled-solo</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>格陵兰犬拉雪橇独行</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>零下三十度，全世界只有你和十二条狗</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>零下三十度，全世界只有你和十二条狗</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>伊卢利萨特冰峡湾的狗拉雪橇不是表演，是唯一的交通方式。向导把缰绳递给你，就回去喝咖啡了。在白茫茫的冰盖上，你必须学会用眼神和吼声指挥犬队，因为迷路在这里的代价是真实的。恐惧和自由在同一个瞬间到来。</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>北极 · 格陵兰</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>extreme</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>raw</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>["极寒";"孤独";"犬队";"生存";"北极"]</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>29999</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>greenland-dog-sled.jpg</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>零下三十度，全世界只有你和十二条狗</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>extreme;solitude;nature</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>ESTP:5;ENTJ:4;ISTP:4</t>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>极限挑战(extreme);孤独感(solitude);自然原始(nature)</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>ESTP-企业家:5;ENTJ-指挥官:4;ISTP-鉴赏家:4</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>norway-aurora-hunt</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>挪威特罗姆瑟极光狩猎</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>在零下二十度的黑夜里，等一束来自太阳的光</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>在零下二十度的黑夜里，等一束来自太阳的光</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>特罗姆瑟的冬天没有白天，只有漫长的蓝调和黑夜。你裹着三层羽绒服躺在雪地上，脖子仰成九十度，等待那道绿色的帷幕从地平线缓缓升起。当极光真正爆发时，整个天空都在跳舞——你会忘记寒冷，忘记时间，甚至忘记自己是谁。</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>欧洲 · 挪威</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>dramatic</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>["极光";"寒冷";"等待";"爆发";"夜空"]</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
         <is>
           <t>18999</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>norway-aurora.jpg</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>在零下二十度的黑夜里，等一束来自太阳的光</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>visual;nature;night</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>INFP:5;ISFJ:4;INFJ:5</t>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>视觉奇观(visual);自然原始(nature);夜晚魔法(night)</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>INFP-调停者:5;ISFJ-守护者:4;INFJ-提倡者:5</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>new-zealand-milford-kayak</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>新西兰米尔福德峡湾皮划艇</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>在两千米高的瀑布下，你渺小得像一滴水</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>在两千米高的瀑布下，你渺小得像一滴水</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>米尔福德峡湾的峭壁从水面直接拔起两千米，岩壁上挂满了临时瀑布——前一秒还是晴天，下一秒暴雨就让几百条银线同时坠入海中。你划着皮划艇靠近其中一条，水雾打在脸上，分不清是雨水、海水还是瀑布的水。</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>大洋洲 · 新西兰</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>extreme</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>raw</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>["瀑布";"皮划艇";"水雾";"渺小";"暴雨"]</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>22999</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>new-zealand-milford.jpg</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>在两千米高的瀑布下，你渺小得像一滴水</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>extreme;visual;nature</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>ENTP:4;ESTP:5;ISTP:5</t>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>极限挑战(extreme);视觉奇观(visual);自然原始(nature)</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>ENTP-辩论家:4;ESTP-企业家:5;ISTP-鉴赏家:5</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>patagonia-torres-del-paine-trek</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>巴塔哥尼亚百内国家公园徒步</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>狂风把云撕碎，露出花岗岩的尖顶</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>狂风把云撕碎，露出花岗岩的尖顶</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>百内国家公园的天气变化比心跳还快。前一秒狂风暴雨，下一秒阳光就把三塔峰照成金色。你背着四十升的包在碎石坡上艰难前行，每一步都在和地心引力谈判。但当W线走完的那一刻，你明白了为什么有人愿意飞三十个小时来受这个罪。</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>南美洲 · 智利</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>extreme</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>dramatic</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>["狂风";"徒步";"花岗岩";"三塔峰";"挑战"]</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t>24999</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>patagonia-torres-del-paine.jpg</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>狂风把云撕碎，露出花岗岩的尖顶</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>extreme;hidden;nature</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>INTJ:5;ISTJ:4;ENTJ:5</t>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>极限挑战(extreme);隐秘小众(hidden);自然原始(nature)</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>INTJ-建筑师:5;ISTJ-物流师:4;ENTJ-指挥官:5</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>turkey-cappadocia-balloon</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>土耳其卡帕多西亚热气球日出</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>一百个热气球同时升空，你漂浮在月球表面</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>一百个热气球同时升空，你漂浮在月球表面</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>凌晨四点半，卡帕多西亚的峡谷还笼罩在蓝调中。火焰喷射器间歇性轰鸣，巨大的彩色球体一个接一个挣脱地心引力。当太阳从地平线跃出，把整个峡谷染成玫瑰金色，你低头看着那些精灵烟囱和洞穴教堂——这是人类最接近飞行梦想的时刻。</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>亚洲 · 土耳其</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>visual</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>surreal</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>["热气球";"日出";"月球";"玫瑰金";"飞行"]</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
         <is>
           <t>16999</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>turkey-cappadocia.jpg</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>一百个热气球同时升空，你漂浮在月球表面</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>visual;culture;night</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>ENFP:5;ISFP:4;ESFP:5</t>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>视觉奇观(visual);文化沉浸(culture);夜晚魔法(night)</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>ENFP-竞选者:5;ISFP-探险家:4;ESFP-表演者:5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>peru-machu-picchu-inca-trail</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>秘鲁马丘比丘印加古道徒步</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>四天三夜，走在五百年前铺好的石阶上</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>四天三夜，走在五百年前铺好的石阶上</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>印加古道不是观光路线，是一次时间旅行。你踩着五百年前印加工匠凿出来的石阶，穿过云雾森林，越过海拔四千二百米的死亡女峰。第四天凌晨，当浓雾突然散开，马丘比丘的轮廓出现在你面前——那一刻，所有的肌肉酸痛都变成了值得。</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>南美洲 · 秘鲁</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>culture</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>["古道";"印加";"石阶";"云雾";"时间"]</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>21999</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>peru-machu-picchu.jpg</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>四天三夜，走在五百年前铺好的石阶上</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>extreme;culture;hidden</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>ISFJ:5;ISTJ:5;INFJ:4</t>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>极限挑战(extreme);文化沉浸(culture);隐秘小众(hidden)</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>ISFJ-守护者:5;ISTJ-物流师:5;INFJ-提倡者:4</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>namibia-deadvlei-stars</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>纳米比亚死亡谷星空露营</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>九百年的枯树站在红沙丘上，像大地竖起的图腾</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>九百年的枯树站在红沙丘上，像大地竖起的图腾</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>死亡谷不是真的死亡——它只是不再下雨。九百年前枯死的骆驼刺树依然站立在龟裂的白色盐沼上，背景是世界上最高的红沙丘。夜晚在附近扎营，没有月亮，银河从沙丘顶端倾泻而下，那些枯树的剪影在星光下像某种远古的仪式现场。</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>非洲 · 纳米比亚</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>surreal</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>["枯树";"红沙丘";"银河";"盐沼";"远古"]</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
         <is>
           <t>19999</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>namibia-deadvlei.jpg</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>九百年的枯树站在红沙丘上，像大地竖起的图腾</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>visual;nature;night</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>INFP:5;INTJ:4;INFJ:5</t>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>视觉奇观(visual);自然原始(nature);夜晚魔法(night)</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>INFP-调停者:5;INTJ-建筑师:4;INFJ-提倡者:5</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>maldives-underwater-dining</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>马尔代夫海底餐厅晚宴</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>在五米深的海底，和鲨鱼一起享用香槟</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>在五米深的海底，和鲨鱼一起享用香槟</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>马尔代夫康拉德酒店的海底餐厅Ithaa，是一个全透明的丙烯酸穹顶。你坐在海底五米处，脚下是白沙和珊瑚，头顶是游过的蝠鲼和礁鲨。侍者端上香槟的那一刻，一条护士鲨恰好从窗外掠过——这是地球上最浪漫的晚餐，没有之一。</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
         <is>
           <t>亚洲 · 马尔代夫</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>visual</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>surreal</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>["海底";"鲨鱼";"香槟";"穹顶";"浪漫"]</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
         <is>
           <t>35999</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>maldives-underwater.jpg</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>在五米深的海底，和鲨鱼一起享用香槟</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>visual;culture;hidden</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>ISFJ:4;ESFJ:5;ENFJ:5</t>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>视觉奇观(visual);文化沉浸(culture);隐秘小众(hidden)</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>ISFJ-守护者:4;ESFJ-执政官:5;ENFJ-主人公:5</t>
         </is>
       </c>
     </row>

</xml_diff>